<commit_message>
UPD - add RNA-seq results OE, shRNA and TDI
</commit_message>
<xml_diff>
--- a/neuroblastoma/results/RNA-seq/RNA-seq_shRNA_pairwise/LUC_DOX_vs_CTRL_fgsea_results.xlsx
+++ b/neuroblastoma/results/RNA-seq/RNA-seq_shRNA_pairwise/LUC_DOX_vs_CTRL_fgsea_results.xlsx
@@ -436,19 +436,19 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.748953974895398</v>
+        <v>0.704545454545455</v>
       </c>
       <c r="C2">
-        <v>0.967032967032967</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D2">
-        <v>0.0611692626746689</v>
+        <v>0.0635007968065945</v>
       </c>
       <c r="E2">
         <v>-0.452924271475521</v>
       </c>
       <c r="F2">
-        <v>-0.749949953771765</v>
+        <v>-0.78275933319936</v>
       </c>
       <c r="G2">
         <v>55</v>
@@ -481,19 +481,19 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.456066945606695</v>
+        <v>0.416161616161616</v>
       </c>
       <c r="C3">
-        <v>0.956880733944954</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D3">
-        <v>0.0865399737444125</v>
+        <v>0.0897104652742981</v>
       </c>
       <c r="E3">
         <v>-0.584995038878827</v>
       </c>
       <c r="F3">
-        <v>-0.971257464579038</v>
+        <v>-1.01262610602188</v>
       </c>
       <c r="G3">
         <v>56</v>
@@ -526,19 +526,19 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.847583643122677</v>
+        <v>0.833941605839416</v>
       </c>
       <c r="C4">
-        <v>0.967032967032967</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D4">
-        <v>0.0498907356726307</v>
+        <v>0.0497903187820785</v>
       </c>
       <c r="E4">
         <v>0.415662777094024</v>
       </c>
       <c r="F4">
-        <v>0.6616831987377</v>
+        <v>0.667218077910773</v>
       </c>
       <c r="G4">
         <v>194</v>
@@ -571,19 +571,19 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.146534653465347</v>
+        <v>0.145418326693227</v>
       </c>
       <c r="C5">
-        <v>0.956880733944954</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D5">
-        <v>0.161978948883402</v>
+        <v>0.163180127180689</v>
       </c>
       <c r="E5">
         <v>-0.822227197429431</v>
       </c>
       <c r="F5">
-        <v>-1.38524242966084</v>
+        <v>-1.36982111885591</v>
       </c>
       <c r="G5">
         <v>21</v>
@@ -616,19 +616,19 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.506958250497018</v>
+        <v>0.525793650793651</v>
       </c>
       <c r="C6">
-        <v>0.956880733944954</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D6">
-        <v>0.0780892306943345</v>
+        <v>0.0760837160951725</v>
       </c>
       <c r="E6">
         <v>-0.587728966010003</v>
       </c>
       <c r="F6">
-        <v>-0.983276551610609</v>
+        <v>-0.982448594627066</v>
       </c>
       <c r="G6">
         <v>20</v>
@@ -661,26 +661,26 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.967032967032967</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="C7">
-        <v>0.967032967032967</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D7">
-        <v>0.051530912208539</v>
+        <v>0.0438002031299891</v>
       </c>
       <c r="E7">
-        <v>-0.394317220740825</v>
+        <v>0.411268673651387</v>
       </c>
       <c r="F7">
-        <v>-0.59438113152195</v>
+        <v>0.620940629097672</v>
       </c>
       <c r="G7">
-        <v>839</v>
+        <v>858</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>FAM72D; HDDC2; NUAK2; WWC1; KCNB1; MCM10; MKI67; CDCA3; EXOSC9; KAZN; FAM122B; CIT; RPS6KA6; ARL13B; GTF2H2; BCYRN1; HSPA14; RAP1GDS1; RBM14; FP565260.1; TNFSF18; NIPAL4; MYBL1; CDC6; DIAPH3; RASSF2; ATAD2; TBCE; NCAPG2; TXNRD2; CEP55; AMD1; PPAT; CCNA2; RRS1; RIPK2; PLAU; MALT1; PCID2; DFFA; NOP58; FH; TK1; UGDH; NOL11; MBD2; PCGF5; UHRF1; NOP14; ALDH1B1; DGKD; WDR43; SCIN; GNPNAT1; ARHGAP29; SHROOM3; HS6ST1; CSRP1; YARS1; LARP4; TMEM237; BCCIP; MRPL3; PRR11; CLDN1; PTGES3; ZBTB18; DAB2; TCOF1; VKORC1L1; RNF41; SIRPA; MYBBP1A; ADGRG6; ETS1; DDAH1; NOL6; PTPN14; MAML2; UBE2J1; ANLN; GNAI1; SRF; ELAVL1; MYC; MID1; ALPK2; CLIP1; EIF4E; DUSP14; EIF2S2; EHD1; PHLDB2; CSE1L; FLNC; BCL7A; SMS; ARSJ; KPNA3; AFAP1; ARHGAP18; LRRC59; ANKRD52; KIF5B; NEK7; LATS2; RGMB; SLC7A5; ARID5B; CCN2; PAICS; SPTLC2; NEDD9; CAVIN1; CCN1; SH3BP4; ATP8B1; FBN2; ADAM19; LIMA1; RAD23B; LASP1; GNG12; ST3GAL5; MATN2; SRSF2; IPO5; MCAM; ASPH; PSAT1; NCL; RSL1D1; THBS1; CUL4B; TUBA1B; ENO1; SERPINE2; MARCHF4; PADI2; RCAN1; GSPT1; LBH; TUBB; SEPTIN11; SRSF1; STIP1; MYO1C; FGF2; PSMD2; CDV3; TRAM2; CCT4; TARS1; BCAR1; DDX21; HSP90AA1; ANXA5; TFRC; DDR2; TAX1BP3; COTL1; INHBA; GALNT10; MAPRE1; ADAM9; HSPA8; TGFB2; ACTB; PFKP; ANKRD1; CITED2; LOXL2; C1orf198; VDAC1; CAP1; TUBB4B; TOM1L2; NUAK1; ANXA1; BASP1; KPNA2</t>
+          <t>OIP5; LAMA3; GABRA5; FAM72B; ARNTL2; MT2A; HACD1; NDUFAF2; ARHGAP23; SKP2; UBE2C; FLNB; MNAT1; NOP16; UCP2; NDUFAF4; UGP2; MATR3; NTMT1; RAN; PPP2R2A; SNU13; AP1S3; EMG1; DDX47; PIEZO1; SNRPG; CCDC85C; CDK2; RPL26L1; BYSL; MIR4435-2HG; TUFT1; LMO7; UBE2S; MPP5; INTS13; IQCJ-SCHIP1; GLIPR2; RANGAP1; HAUS6; EIF2S1; DCAF13; RPL22L1; PRELID1; PSMD11; AJUBA; PAWR; UBASH3B; BMP2K; RRP7A; TIMM50; ADK; RDH10; ARHGAP11A; G3BP1; COPS6; SLC2A1; RRM1; PRC1; NF2; CLPTM1L; CPA4; EVA1A; PIP5K1A; SLC16A3; DKK1; MAP2K3; SSR3; ELL2; NSD2; NAA15; RANBP1; SRSF3; USP53; HSPE1; TUBA1C; LSM12; SPCS3; MEST; GTPBP4; MME; ERCC2; MBNL1; HSPA4; CYB5B; CCT6A; MTHFD2; ANKRD13A; LDHA; TMSB4X; PSG5; HNRNPH3; EPAS1; TPM1; FSTL1; EIF1AX; C12orf75; PEA15; H2AZ1; S100A10; LMNB2; PGRMC2; FRMD6; ACTN4; PRPS1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -706,26 +706,26 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.546788990825688</v>
+        <v>0.806521739130435</v>
       </c>
       <c r="C8">
-        <v>0.956880733944954</v>
+        <v>0.964814814814815</v>
       </c>
       <c r="D8">
-        <v>0.070113215764256</v>
+        <v>0.059476028695732</v>
       </c>
       <c r="E8">
-        <v>0.609123241626482</v>
+        <v>-0.460773772030888</v>
       </c>
       <c r="F8">
-        <v>0.919624837159694</v>
+        <v>-0.696451746787489</v>
       </c>
       <c r="G8">
-        <v>842</v>
+        <v>871</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TRIM73; ANKRD44; DICER1-AS1; WNT11; SBK1; SHD; KLHL3; LINC02691; YPEL1; STK16; HEXD; CASTOR3; GLI4; ELAVL2; MANSC1; ATP8A1; PPP1R13B; PHETA1; DGLUCY; OSBPL7; GMIP; KIF5A; LMBR1L; AC068580.4; RASA4; BCAS3; KLF13; PLCB4</t>
+          <t>FP236383.3; ADAM22; GTF2IP1; MAML3; CYGB; SMAD9; EML5; KCNH5; BTN3A3; RASA4B; SAMD9</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">

</xml_diff>